<commit_message>
updated excel for data migration
</commit_message>
<xml_diff>
--- a/data/migration/invert_data_migration_to_new_excel.xlsx
+++ b/data/migration/invert_data_migration_to_new_excel.xlsx
@@ -12496,7 +12496,7 @@
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -12524,7 +12524,7 @@
       </c>
       <c r="G506" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -12552,7 +12552,7 @@
       </c>
       <c r="G507" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -12580,7 +12580,7 @@
       </c>
       <c r="G508" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -12608,7 +12608,7 @@
       </c>
       <c r="G509" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -12636,7 +12636,7 @@
       </c>
       <c r="G510" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -20708,7 +20708,7 @@
       </c>
       <c r="G834" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -20736,7 +20736,7 @@
       </c>
       <c r="G835" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4</t>
         </is>
       </c>
     </row>

</xml_diff>